<commit_message>
chasers and bug fixes
</commit_message>
<xml_diff>
--- a/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcc86d9586698491e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R14c5cfa286d746d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R96191e09dea14a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R746b33da035f411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rfe98a6edb6964ff1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R3b8e4f9365d14b13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R1b6167c7f8ee4fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R4d28c3fb74694c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Red671b4d6beb47db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rc8fbcba9b0304743"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R2bfb5926385f48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R146aa5d17e674aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R5970563b55154c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5e89322b57934766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R6f4760134a0a47b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R8e9588920f084747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R43421266426f4323"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R078df61baac64514"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R6d868e37bab54ae3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rf97cb9494d234408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R04dde9cca1cb42da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R4416ec132511442d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R5a47c0d7efb34093"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rcfe088a08840494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rcfba3874cbbb4679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R6ddcb59ede384b2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2101,7 +2101,7 @@
         <x:v>Right-bank completion arms first post-reset drop to expand moving window 1 -&gt; 2 -&gt; 3; STAR freezes current window 10s/15s</x:v>
       </x:c>
       <x:c r="L21" s="31" t="str">
-        <x:v>One shipment, or two with More Jackpots / ball end</x:v>
+        <x:v>Three shipments, or four with More Jackpots / ball end</x:v>
       </x:c>
       <x:c r="M21" s="31" t="str">
         <x:v>Crime Wave risk/reward chase. Availability now grows through the approved one-, two-, and three-saucer moving windows. Only red hole lamps show valid saucers; scoring, chase speeds, Diamond Bonus, Case Files, red STAR flash, and terminal summary hold remain intact.</x:v>
@@ -2417,18 +2417,16 @@
         </x:is>
       </x:c>
       <x:c r="J27" s="31" t="str">
-        <x:v>Five chances; three correct required. More JP gives seven chances. Correct: 100K base, +50K each; Bigger JP: 150K base, +75K each. Wrong: 10K.</x:v>
+        <x:v>Four rounds; four correct required. More JP adds two recovery rounds. Clean JPs 200K/300K/400K/500K; first wrong -100K and removes that choice. Bigger: 300K/450K/600K/750K with -150K first-wrong penalty.</x:v>
       </x:c>
       <x:c r="K27" s="31" t="str">
-        <x:v>Lens-safe green indicators avoid weak red output through green bank inserts. Result GI restores after 350ms, and l_gi_a remains in the normal Pardo GI theme.</x:v>
+        <x:v>All live choices flash green identically. Reveal isolates the correct flashing choice. Summary tracks first-guess and second-guess Jackpots.</x:v>
       </x:c>
       <x:c r="L27" s="31" t="str">
-        <x:v>Third correct shot or final available chance</x:v>
-      </x:c>
-      <x:c r="M27" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mystic chapter reveal/mistake-limit role.</x:t>
-        </x:is>
+        <x:v>Fourth correct Jackpot or final available recovery round</x:v>
+      </x:c>
+      <x:c r="M27" s="31" t="str">
+        <x:v>Mystic chapter reveal/mistake-limit role.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -8538,7 +8536,7 @@
         </x:is>
       </x:c>
       <x:c r="G27" s="31" t="str">
-        <x:v>Implemented / recent spinner lighting fix</x:v>
+        <x:v>Four base rounds; More JP adds two recovery rounds. Each round presents three choices selected from seven logical shot groups; the three upper targets are one shared choice. All currently available choices flash green identically. Spinner reveals the correct choice for 4s, or 6s with More Time: the correct choice flashes and wrong choices go dark. First wrong scores 20K, removes that choice, and reduces the current Jackpot; the remaining two resume flashing. Second wrong loses the round. Four correct Jackpots defeat Pardo. Summary counts 1st-guess JPs and 2nd-guess JPs.</x:v>
       </x:c>
       <x:c r="H27" s="31" t="str">
         <x:v>Five chances, or seven with More JP. Each chance presents three choices selected from seven logical shot groups; the three upper targets are one shared upper-target group so they can never show conflicting good/bad states. Spinner reveals the correct choice for 4s, or 6s with More Time. Three correct shots defeats Pardo immediately. Using all chances with fewer than three correct shots produces the escape result. Hidden choices use solid green for white/green lens compatibility; reveal flashes only the correct green choice and turns wrong choices off. The main spinner insert flashes white while choices are hidden, turns off during the reveal, and resumes if another reveal is needed. Result GI flashes for 350ms, then restores.</x:v>
@@ -11885,7 +11883,7 @@
         <x:v>Build the Frozen Diamond Jackpot with both drop banks. Any right drop starts a moving one-saucer shipment window. Complete/reset the right bank, then hit the first post-reset right drop to expand the moving window to two saucers; repeat to reach three.</x:v>
       </x:c>
       <x:c r="G21" s="31" t="str">
-        <x:v>Collect one correct saucer shipment, or two with More Jackpots; otherwise stops on ball end. A terminal saucer remains held until the villain summary ends.</x:v>
+        <x:v>Collect three correct saucer shipments, or four with More Jackpots; otherwise stops on ball end. A terminal saucer remains held until the villain summary ends.</x:v>
       </x:c>
       <x:c r="H21" s="31" t="str">
         <x:v>Drops score 25K and bank 25K Diamond Bonus. Base Jackpot is 100K; right drops add 25K and left drops add 40K. Bigger uses 200K/+50K/+75K. Wrong saucer scores 10K. STAR banks 100K and freezes the current available window for 10s/15s.</x:v>
@@ -12112,16 +12110,16 @@
         </x:is>
       </x:c>
       <x:c r="F27" s="31" t="str">
-        <x:v>Find the correct shot among three choices and collect three Hypnosis Jackpots before the available chances expire.</x:v>
+        <x:v>Find the correct shot among three flashing choices. The spinner reveals the answer; four correct Hypnosis Jackpots defeat Pardo.</x:v>
       </x:c>
       <x:c r="G27" s="31" t="str">
-        <x:v>Third correct shot defeats Pardo; fewer than three correct after five chances (seven with More JP) lets him escape.</x:v>
+        <x:v>Four correct Jackpots defeat Pardo. Four base rounds are available; More Jackpots adds two recovery rounds.</x:v>
       </x:c>
       <x:c r="H27" s="31" t="str">
-        <x:v>Spinner reveals the correct choice for 4 seconds (6 seconds with More Time). Correct Jackpots start at 100K and increase 50K; Bigger JP starts at 150K and increases 75K. Wrong choices score 10K and consume the chance.</x:v>
+        <x:v>Normal clean Jackpot ladder: 200K/300K/400K/500K. One wrong choice reduces the current Jackpot by 100K. Bigger uses 300K/450K/600K/750K with a 150K first-wrong reduction. Every wrong choice scores 20K. Reveal is 4s, or 6s with More Time.</x:v>
       </x:c>
       <x:c r="I27" s="31" t="str">
-        <x:v>Seven logical shot groups; three are selected per chance. Upper-left, upper-center, and upper-right targets are one grouped choice and always share the same good/bad state. Hidden choices are solid green across white and green lenses. Reveal flashes only the correct choice green and turns wrong choices off. Result GI restores after a 350ms green/red confirmation. Shot Assist makes all three choices correct on the first chance. Summary outcome distinguishes defeat from escape.</x:v>
+        <x:v>Seven logical shot groups; three selected per round. Upper-left/center/right targets are one grouped choice. Available choices flash green identically; first wrong goes dark and the two survivors continue flashing. Spinner reveal flashes only the correct choice and turns wrong choices off. Shot Assist makes all three choices correct in Round 1. Summary stats are 1ST-GUESS JPs and 2ND-GUESS JPs.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
fixes and chapter music fix
</commit_message>
<xml_diff>
--- a/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc15563cc366a45d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rcb48084f83934f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Ref5787e6098049dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R88cf85b24a634a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R665d7239060c4d42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R3512c3331cc34379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R063b5a35b1f74514"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R9a0ed0fa7ba94b5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R20dce9fe8f084082"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R0551c8de669a4645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Ref30b921f7bc4abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rac489fc127304a0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R7128a9b49bde4212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R577f5063c1424653"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rb78b5da84916494c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rf8ddf1207e7f411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R4aad6d1e67b44403"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rcbc240de532f4271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Rbc7045f4109642ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rbe51306fc7c245d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R81e58da296bb412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rc6ac95a55dc9403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R2f5e92ee87a6499a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rae56216b45f8419e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rfae4cb7ac8d84e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Raab6976be78c4010"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9538,10 +9538,8 @@
           <x:t xml:space="preserve">Implemented / needs playtest</x:t>
         </x:is>
       </x:c>
-      <x:c r="H50" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Complete all eight lower drops in strict left-to-right order. Each upper-spinner spin drops the next required target; the player may advance directly only by hitting that same target. A wrong direct hit resets only that bank, then restores completed targets after 200ms with 200ms staged re-drops. Correct drops score 100K. Completing all eight lights a 15s center-web Super for 500K; expiry ends the one allowed attempt.</x:t>
-        </x:is>
+      <x:c r="H50" s="31" t="str">
+        <x:v>Complete all eight lower drops in strict left-to-right order. Each upper-spinner spin drops the next required target; the player may advance directly only by hitting that same target. A wrong direct hit resets only that bank, then restores completed targets after 200ms with 200ms staged re-drops. Correct drops score 100K. Completing all eight lights a 20s center-web Super for 500K; expiry ends the one allowed attempt. More Time extends the Super window to 25s.</x:v>
       </x:c>
       <x:c r="I50" s="31" t="inlineStr">
         <x:is>
@@ -13049,15 +13047,11 @@
       <x:c r="F50" s="31" t="str">
         <x:v>Complete left 1-3, then right 1-5 in order. After the startup bank reset, the rooftop gate opens and remains open while the upper spinner is needed; each spin drops the next target. A correct direct hit also advances. A wrong direct hit resets only that bank and restores its completed targets after 200ms, with 200ms staged re-drops.</x:v>
       </x:c>
-      <x:c r="G50" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">After all eight drops, the center web is lit for 15s. Center Super defeats Skymaster. Expiry ends the mode unsuccessfully with no second attempt. More Jackpots also lights the left web; each web can score once.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H50" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Correct drops 100K; center/left web Supers 500K. Bigger: 150K drops and 750K Supers. More Time: 20s. Safety: opening 10s save. Assist: first upper spin advances two drops.</x:t>
-        </x:is>
+      <x:c r="G50" s="31" t="str">
+        <x:v>After all eight drops, the center web is lit for 20s. Center Super defeats Skymaster. Expiry ends the mode unsuccessfully with no second attempt. More Jackpots also lights the left web; each web can score once.</x:v>
+      </x:c>
+      <x:c r="H50" s="31" t="str">
+        <x:v>Correct drops 100K; center/left web Supers 500K. Bigger: 150K drops and 750K Supers. More Time: 25s. Safety: opening 10s save. Assist: first upper spin advances two drops.</x:v>
       </x:c>
       <x:c r="I50" s="31" t="str">
         <x:v>Implemented with all eight physical drop coils, programmatic-switch guards, strict direct-hit validation, 200ms bank restoration staging, explicit ordered-phase rooftop gate ownership, VUK shared eject handling, gate closure for the Web Super and mode stop, target/web lighting, one-attempt timer, Case Files, status, and summary values; needs on-machine playtest.</x:v>

</xml_diff>

<commit_message>
web tightens wiz mode
</commit_message>
<xml_diff>
--- a/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R577f5063c1424653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rb78b5da84916494c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rf8ddf1207e7f411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R4aad6d1e67b44403"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rcbc240de532f4271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Rbc7045f4109642ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rbe51306fc7c245d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R81e58da296bb412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rc6ac95a55dc9403c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R2f5e92ee87a6499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rae56216b45f8419e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rfae4cb7ac8d84e23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Raab6976be78c4010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5009715350984401"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R81f3362f526042a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R8dbac9c2fe23481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rbc5eca579f3f4a1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R55a416502bc14687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Red00f9f479dc423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Ra7c50e6d665c4a30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rb276d363099f4086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R128807cc11b849ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rd1a7538ae97f439b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R7b4dba70370a4bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rc8bfe6ba1e9d4b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Rf78e46a40b4847c3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4846,10 +4846,8 @@
           <x:t xml:space="preserve">The Web Tightens</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Placeholder shell — full design/coding required</x:t>
-        </x:is>
+      <x:c r="E6" s="31" t="str">
+        <x:v>Approved/coded — needs playtest</x:v>
       </x:c>
       <x:c r="F6" s="85" t="n"/>
       <x:c r="G6" s="85" t="n"/>
@@ -10043,15 +10041,11 @@
           <x:t xml:space="preserve">start_mode_the_web_tightens</x:t>
         </x:is>
       </x:c>
-      <x:c r="F6" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G6" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
+      <x:c r="F6" s="31" t="str">
+        <x:v>No individual Case File powers. Each 1X phase Jackpot = 100K + 20K × the chapter's collected Case Files (0–25 files; +0–500K). 2X phase Jackpots double both base and prep. The rooftop Super is separate at 1M × successful phases and does not receive Wizard Prep.</x:v>
+      </x:c>
+      <x:c r="G6" s="31" t="str">
+        <x:v>Approved/coded from the 2026-09-01 design: repeating 2-ball/VUK-lock wizard with Fiddler, Metal-Eating Monster, Conquistador, Spider-Slayer, and Harley &amp; Clivendon phases; saucers park excess balls; Chapter Case Files add 20K to every 1X phase JP; phase wins build a 1M-per-success rooftop Super. Needs machine playtest and polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -13545,10 +13539,8 @@
           <x:t xml:space="preserve">Playtest coded mini-wizards</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sinister Surge and Trubble Unleashed are approved/coded. Mastermind Trap, Crime Wave, and Fifth Dimension Curse are functional but provisional and require design approval as well as playtest.</x:t>
-        </x:is>
+      <x:c r="C2" s="45" t="str">
+        <x:v>Sinister Surge, Trubble Unleashed, and The Web Tightens are approved/coded. Mastermind Trap, Crime Wave, and Fifth Dimension Curse are functional but provisional and require design approval as well as playtest.</x:v>
       </x:c>
       <x:c r="D2" s="45" t="inlineStr">
         <x:is>
@@ -13795,10 +13787,8 @@
           <x:t xml:space="preserve">Finish mini-wizard and final-wizard designs</x:t>
         </x:is>
       </x:c>
-      <x:c r="C14" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Review 3 functional/provisional mini-wizards; fully design and code 6 placeholder shells; complete the dedicated Kingpin Final Showdown design/retheme. Wizard Case Files add only 20K each to Jackpot/Super Jackpot values (max +500K).</x:t>
-        </x:is>
+      <x:c r="C14" s="45" t="str">
+        <x:v>Review 3 functional/provisional mini-wizards; fully design and code 5 remaining placeholder shells; complete the dedicated Kingpin Final Showdown design/retheme. The Web Tightens is approved/coded and needs machine playtest. Wizard Case Files add 20K each to qualifying Jackpot values (max +500K per 1X JP).</x:v>
       </x:c>
       <x:c r="D14" s="45" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
fiddler stuff for wiz mode
</commit_message>
<xml_diff>
--- a/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R88c0d65645a04647"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R7cceebe8494545cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R9858b8b3a2de4f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R200a28cd274a4847"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R6128c5b3700a4feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Rb37a130f22ce43b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rad88e0472a93495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Red4dfe5e86754295"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R65e4513eb899455d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rce5f05f276754c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R75796648cadc42fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Ref5bf6f925a94378"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R025df34039ce473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R473a536312b44f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R3d76a2671dd64356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R23bc86742f6d4bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R5f6517ccc24048a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R8119b5e63cf245b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R3ce2bbb22eda4524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Reb1cf4162c9741ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rab62ab6def1a4b2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rb0c775df06874376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R090ebaedf6474bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R8b3956aa187445fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R6df9b7d243b447ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R7c633ec0ec874d17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10015,7 +10015,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="132" hidden="0" customHeight="1">
       <x:c r="A6" s="31" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -10043,7 +10043,7 @@
         <x:v>No individual Case File powers. Each 1X phase Jackpot = 100K + 20K × the chapter's collected Case Files (0–25 files; +0–500K). 2X phase Jackpots double both base and prep. The rooftop Super is separate at 1M × successful phases and does not receive Wizard Prep.</x:v>
       </x:c>
       <x:c r="G6" s="31" t="str">
-        <x:v>Approved/coded from the 2026-09-01 design: repeating 2-ball/VUK-lock wizard with Fiddler, Metal-Eating Monster, Conquistador, Spider-Slayer, and Harley &amp; Clivendon phases; saucers park excess balls; Chapter Case Files add 20K to every 1X phase JP; phase wins build a 1M-per-success rooftop Super. Needs machine playtest and polish.</x:v>
+        <x:v>Approved/coded from the 2026-09-01 design: repeating 2-ball/VUK-lock wizard with Fiddler, Metal-Eating Monster, Conquistador, Spider-Slayer, and Harley &amp; Clivendon phases; saucers park excess balls; Chapter Case Files add 20K to every 1X phase JP; phase wins build a 1M-per-success rooftop Super. Needs machine playtest and polish. Fiddler parity update: both drop banks stage down during GET READY; individual drop switches are ignored; the exposed left/right bank rubbers are the bank-note inputs; WATCH strobe, note gaps, repeat pause, and correct/wrong feedback match standalone Fiddler.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
ball save, daily, centaur, etc
</commit_message>
<xml_diff>
--- a/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R473a536312b44f7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R3d76a2671dd64356"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R23bc86742f6d4bf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R5f6517ccc24048a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R8119b5e63cf245b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R3ce2bbb22eda4524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Reb1cf4162c9741ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rab62ab6def1a4b2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rb0c775df06874376"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R090ebaedf6474bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R8b3956aa187445fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R6df9b7d243b447ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R7c633ec0ec874d17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R34f31d7c8aab4a10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rea01e5faef9f4f61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R4658386001564602"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R71bad4fed899403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Ref9a1f1d09734add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R5ae247d37f9a47ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rdd8adb27d024428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rf269164e7ae3430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R99b7be21bbcf4bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Reb8b6bad867c43bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R5783142f535948cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R4e4cfa79d51649ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R815fd955cc344958"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10103,15 +10103,11 @@
           <x:t xml:space="preserve">start_mode_mad_science_meltdown</x:t>
         </x:is>
       </x:c>
-      <x:c r="F8" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G8" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
+      <x:c r="F8" s="31" t="str">
+        <x:v>No individual Case File powers. Every Gas and Noah Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Red/yellow gas awards, upper-spinner build increments, and the 1M four-ball Magneto award do not receive this bonus.</x:v>
+      </x:c>
+      <x:c r="G8" s="31" t="str">
+        <x:v>Approved/coded: repeating 3-ball multiball with 20s opening save. Each left drop releases one independent gas zone; lower-spinner hits cool all active zones red → yellow → green; green collects a 500K+ Case File Gas Jackpot. Upper targets and early right-drop hits eliminate Noah's false locations; the last standing right target collects a 500K+ Case File + 100K-per-upper-spin Noah Jackpot. Saucers park up to two balls for 2X/3X Noah and release on collect. Middle A+B lights center web for 10s: Add-a-Ball with 10s save below four balls, otherwise 1M. No final objective; ends when multiball ends. Needs machine playtest and presentation polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>